<commit_message>
Fix remaining folder name strings in test steps
</commit_message>
<xml_diff>
--- a/test-plans/Test_Cases_Signup_Authorized_Partner.xlsx
+++ b/test-plans/Test_Cases_Signup_Authorized_Partner.xlsx
@@ -1624,7 +1624,7 @@
       </c>
       <c r="E23" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Simulate failure
-2. Check screenshots folder
+2. Check bug-reports folder
 3. Verify file created
 4. Verify screenshot shows error</v>
       </c>
@@ -1678,7 +1678,7 @@
       <c r="E24" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Run npm run test:mocha
 2. Wait for completion
-3. Check test-results folder
+3. Check test-reports folder
 4. Open index.html
 5. Verify report contents</v>
       </c>

</xml_diff>